<commit_message>
feat: refine notifications and control panel
</commit_message>
<xml_diff>
--- a/assets/t-school-control-panel-template.xlsx
+++ b/assets/t-school-control-panel-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="控制臺" sheetId="1" r:id="Raa02139132da4396"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="操作說明" sheetId="2" r:id="R54f1d880918c4eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="控制臺" sheetId="1" r:id="R8754801e884145bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="操作說明" sheetId="2" r:id="R33d5d94686c54d16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -661,7 +661,7 @@
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
       <x:c r="A5" s="17" t="str">
-        <x:v>尚未安裝｜請依下方三個步驟貼上 Code.gs。安裝完成後，所有設定都從上方「行程同步」選單開啟。</x:v>
+        <x:v>尚未安裝｜請依下方三個步驟貼上 Code.gs。安裝完成後，所有設定都從上方「T-SCHOOL Schedule Sync」選單開啟。</x:v>
       </x:c>
       <x:c r="B5" s="18"/>
       <x:c r="C5" s="18"/>
@@ -754,7 +754,7 @@
       </x:c>
       <x:c r="C16" s="29"/>
       <x:c r="D16" s="35" t="str">
-        <x:v>回到這份試算表重新整理，選擇「行程同步 → 開啟設定」。</x:v>
+        <x:v>回到這份試算表重新整理，選擇「T-SCHOOL Schedule Sync → 開啟控制臺介面」。</x:v>
       </x:c>
       <x:c r="E16" s="35"/>
       <x:c r="F16" s="35"/>
@@ -785,7 +785,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="50" t="str">
-        <x:v>行程同步 → 開啟設定</x:v>
+        <x:v>T-SCHOOL Schedule Sync → 開啟控制臺介面</x:v>
       </x:c>
       <x:c r="B22" s="51"/>
       <x:c r="C22" s="51"/>
@@ -899,7 +899,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="68" t="str">
-        <x:v>儲存格不是設定介面；日常操作請一律使用「行程同步」選單與右側控制臺。</x:v>
+        <x:v>儲存格不是設定介面；日常操作請一律使用「T-SCHOOL Schedule Sync」選單與右側控制臺。</x:v>
       </x:c>
       <x:c r="B3" s="68"/>
       <x:c r="C3" s="68"/>
@@ -930,7 +930,7 @@
         <x:v>貼上完整 Code.gs、儲存，然後重新整理試算表。</x:v>
       </x:c>
       <x:c r="D6" s="80" t="str">
-        <x:v>上方出現「行程同步」選單</x:v>
+        <x:v>上方出現「T-SCHOOL Schedule Sync」選單</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="40.5" customHeight="1">
@@ -938,7 +938,7 @@
         <x:v>開啟控制臺</x:v>
       </x:c>
       <x:c r="B7" s="81" t="str">
-        <x:v>行程同步 → 開啟設定</x:v>
+        <x:v>T-SCHOOL Schedule Sync → 開啟控制臺介面</x:v>
       </x:c>
       <x:c r="C7" s="81" t="str">
         <x:v>確認年級、課程、通知與專用日曆。</x:v>
@@ -980,7 +980,7 @@
         <x:v>查看狀態</x:v>
       </x:c>
       <x:c r="B10" s="82" t="str">
-        <x:v>行程同步選單</x:v>
+        <x:v>T-SCHOOL Schedule Sync 選單</x:v>
       </x:c>
       <x:c r="C10" s="82" t="str">
         <x:v>開啟同步狀態或手動執行同步。</x:v>

</xml_diff>